<commit_message>
Renamed the power bi file
</commit_message>
<xml_diff>
--- a/Part_2_EDA/Test Data analyst.xlsx
+++ b/Part_2_EDA/Test Data analyst.xlsx
@@ -8,17 +8,28 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iebs-my.sharepoint.com/personal/stephan_pentchev_student_ie_edu/Documents/Term 2/GameLoft Sofia/Part_2_EDA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{EBE2E45B-C466-4045-B691-58EFD309C04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{EBE2E45B-C466-4045-B691-58EFD309C04F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{056BCA0B-057F-4D25-AE81-6EACF2E75511}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1905" yWindow="1905" windowWidth="21600" windowHeight="11280" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>

</xml_diff>